<commit_message>
add domestic guest view
</commit_message>
<xml_diff>
--- a/src/assets/vms/Employee_List.xlsx
+++ b/src/assets/vms/Employee_List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vanthd\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vanthd\Downloads\source\ufe-vms-app\src\assets\vms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62718266-1EF6-4DA9-B614-4B4A80B19D63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460DC583-B2FA-4E83-B902-6206C74ED11A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D56FC14E-A42E-4C63-AC90-60AFD1F2F23B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{D56FC14E-A42E-4C63-AC90-60AFD1F2F23B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -60,13 +60,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -78,7 +84,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -95,15 +101,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF92D050"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -433,37 +445,38 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BF67412-F73A-44DB-9889-B332A21940B4}">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.77734375" customWidth="1"/>
-    <col min="2" max="2" width="16.21875" customWidth="1"/>
-    <col min="3" max="3" width="25.88671875" customWidth="1"/>
-    <col min="4" max="4" width="25.21875" customWidth="1"/>
-    <col min="5" max="5" width="24.109375" customWidth="1"/>
-    <col min="6" max="6" width="27.77734375" customWidth="1"/>
+    <col min="1" max="1" width="31.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="51" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" customWidth="1"/>
+    <col min="5" max="5" width="38.85546875" customWidth="1"/>
+    <col min="6" max="6" width="37.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>